<commit_message>
B1: 2026-04-07 — 114 plays
</commit_message>
<xml_diff>
--- a/daily/2026-04-07.xlsx
+++ b/daily/2026-04-07.xlsx
@@ -9907,10 +9907,10 @@
         <v>13.2</v>
       </c>
       <c r="J2" t="n">
-        <v>1.8</v>
+        <v>1.806</v>
       </c>
       <c r="K2" t="n">
-        <v>1.943</v>
+        <v>1.926</v>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
@@ -10003,10 +10003,10 @@
         <v>0.2</v>
       </c>
       <c r="J4" t="n">
-        <v>2</v>
+        <v>1.926</v>
       </c>
       <c r="K4" t="n">
-        <v>1.758</v>
+        <v>1.806</v>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
@@ -10147,10 +10147,10 @@
         <v>12.1</v>
       </c>
       <c r="J7" t="n">
-        <v>1.877</v>
+        <v>1.87</v>
       </c>
       <c r="K7" t="n">
-        <v>1.877</v>
+        <v>1.87</v>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
@@ -10243,10 +10243,10 @@
         <v>2</v>
       </c>
       <c r="J9" t="n">
-        <v>1.758</v>
+        <v>1.935</v>
       </c>
       <c r="K9" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
@@ -10339,10 +10339,10 @@
         <v>8</v>
       </c>
       <c r="J11" t="n">
-        <v>1.769</v>
+        <v>1.893</v>
       </c>
       <c r="K11" t="n">
-        <v>2</v>
+        <v>1.833</v>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
@@ -10387,7 +10387,7 @@
         <v>2.2</v>
       </c>
       <c r="J12" t="n">
-        <v>1.82</v>
+        <v>1.806</v>
       </c>
       <c r="K12" t="n">
         <v>1.926</v>
@@ -10483,10 +10483,10 @@
         <v>5.2</v>
       </c>
       <c r="J14" t="n">
-        <v>1.98</v>
+        <v>2</v>
       </c>
       <c r="K14" t="n">
-        <v>1.769</v>
+        <v>1.758</v>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
@@ -10531,10 +10531,10 @@
         <v>2</v>
       </c>
       <c r="J15" t="n">
-        <v>1.735</v>
+        <v>1.769</v>
       </c>
       <c r="K15" t="n">
-        <v>2.02</v>
+        <v>1.98</v>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
@@ -10627,10 +10627,10 @@
         <v>1.4</v>
       </c>
       <c r="J17" t="n">
-        <v>1.735</v>
+        <v>1.952</v>
       </c>
       <c r="K17" t="n">
-        <v>2.02</v>
+        <v>1.787</v>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
@@ -10723,10 +10723,10 @@
         <v>4.1</v>
       </c>
       <c r="J19" t="n">
-        <v>1.769</v>
+        <v>1.758</v>
       </c>
       <c r="K19" t="n">
-        <v>1.98</v>
+        <v>2</v>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
@@ -10915,10 +10915,10 @@
         <v>5.5</v>
       </c>
       <c r="J23" t="n">
-        <v>1.943</v>
+        <v>1.909</v>
       </c>
       <c r="K23" t="n">
-        <v>1.787</v>
+        <v>1.826</v>
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
@@ -11299,10 +11299,10 @@
         <v>1.8</v>
       </c>
       <c r="J31" t="n">
-        <v>1.99</v>
+        <v>2</v>
       </c>
       <c r="K31" t="n">
-        <v>1.781</v>
+        <v>1.769</v>
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
@@ -11347,10 +11347,10 @@
         <v>1.6</v>
       </c>
       <c r="J32" t="n">
-        <v>1.926</v>
+        <v>3.05</v>
       </c>
       <c r="K32" t="n">
-        <v>1.833</v>
+        <v>1.357</v>
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
@@ -11395,10 +11395,10 @@
         <v>1.9</v>
       </c>
       <c r="J33" t="n">
-        <v>1.847</v>
+        <v>1.8</v>
       </c>
       <c r="K33" t="n">
-        <v>1.909</v>
+        <v>1.952</v>
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
@@ -11443,10 +11443,10 @@
         <v>0.5</v>
       </c>
       <c r="J34" t="n">
-        <v>1.943</v>
+        <v>2.75</v>
       </c>
       <c r="K34" t="n">
-        <v>1.82</v>
+        <v>1.417</v>
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
@@ -11491,10 +11491,10 @@
         <v>3.7</v>
       </c>
       <c r="J35" t="n">
-        <v>1.952</v>
+        <v>2</v>
       </c>
       <c r="K35" t="n">
-        <v>1.8</v>
+        <v>1.769</v>
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
@@ -11539,10 +11539,10 @@
         <v>2</v>
       </c>
       <c r="J36" t="n">
-        <v>2.04</v>
+        <v>2.9</v>
       </c>
       <c r="K36" t="n">
-        <v>1.741</v>
+        <v>1.385</v>
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
@@ -11587,10 +11587,10 @@
         <v>2</v>
       </c>
       <c r="J37" t="n">
-        <v>1.87</v>
+        <v>2.8</v>
       </c>
       <c r="K37" t="n">
-        <v>1.893</v>
+        <v>1.408</v>
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
@@ -11635,10 +11635,10 @@
         <v>2.4</v>
       </c>
       <c r="J38" t="n">
-        <v>1.909</v>
+        <v>2.75</v>
       </c>
       <c r="K38" t="n">
-        <v>1.847</v>
+        <v>1.417</v>
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
@@ -11683,10 +11683,10 @@
         <v>1.8</v>
       </c>
       <c r="J39" t="n">
-        <v>1.833</v>
+        <v>2.7</v>
       </c>
       <c r="K39" t="n">
-        <v>1.926</v>
+        <v>1.435</v>
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
@@ -11731,10 +11731,10 @@
         <v>3.3</v>
       </c>
       <c r="J40" t="n">
-        <v>1.877</v>
+        <v>3.05</v>
       </c>
       <c r="K40" t="n">
-        <v>1.877</v>
+        <v>1.357</v>
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
@@ -11779,10 +11779,10 @@
         <v>1.9</v>
       </c>
       <c r="J41" t="n">
-        <v>1.909</v>
+        <v>2.7</v>
       </c>
       <c r="K41" t="n">
-        <v>1.847</v>
+        <v>1.435</v>
       </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
@@ -11827,10 +11827,10 @@
         <v>1.1</v>
       </c>
       <c r="J42" t="n">
-        <v>1.847</v>
+        <v>1.833</v>
       </c>
       <c r="K42" t="n">
-        <v>1.909</v>
+        <v>1.926</v>
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
@@ -11875,10 +11875,10 @@
         <v>0.4</v>
       </c>
       <c r="J43" t="n">
-        <v>1.833</v>
+        <v>3.05</v>
       </c>
       <c r="K43" t="n">
-        <v>1.926</v>
+        <v>1.357</v>
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
@@ -11923,10 +11923,10 @@
         <v>2.8</v>
       </c>
       <c r="J44" t="n">
-        <v>1.952</v>
+        <v>3.05</v>
       </c>
       <c r="K44" t="n">
-        <v>1.813</v>
+        <v>1.357</v>
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
@@ -12643,10 +12643,10 @@
         <v>6.8</v>
       </c>
       <c r="J59" t="n">
-        <v>1.877</v>
+        <v>2.8</v>
       </c>
       <c r="K59" t="n">
-        <v>1.855</v>
+        <v>1.408</v>
       </c>
       <c r="L59" s="2" t="inlineStr">
         <is>
@@ -12691,10 +12691,10 @@
         <v>4</v>
       </c>
       <c r="J60" t="n">
-        <v>1.855</v>
+        <v>3.05</v>
       </c>
       <c r="K60" t="n">
-        <v>1.877</v>
+        <v>1.357</v>
       </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
@@ -12739,10 +12739,10 @@
         <v>9</v>
       </c>
       <c r="J61" t="n">
-        <v>1.847</v>
+        <v>3.1</v>
       </c>
       <c r="K61" t="n">
-        <v>1.885</v>
+        <v>1.345</v>
       </c>
       <c r="L61" s="2" t="inlineStr">
         <is>
@@ -12931,10 +12931,10 @@
         <v>2.7</v>
       </c>
       <c r="J65" t="n">
-        <v>1.885</v>
+        <v>2.75</v>
       </c>
       <c r="K65" t="n">
-        <v>1.847</v>
+        <v>1.417</v>
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
@@ -13027,10 +13027,10 @@
         <v>7.1</v>
       </c>
       <c r="J67" t="n">
-        <v>1.87</v>
+        <v>2.85</v>
       </c>
       <c r="K67" t="n">
-        <v>1.87</v>
+        <v>1.4</v>
       </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
@@ -13078,7 +13078,7 @@
         <v>1.926</v>
       </c>
       <c r="K68" t="n">
-        <v>1.82</v>
+        <v>1.806</v>
       </c>
       <c r="L68" s="2" t="inlineStr">
         <is>
@@ -13363,7 +13363,7 @@
         <v>0.2</v>
       </c>
       <c r="J74" t="n">
-        <v>1.909</v>
+        <v>1.893</v>
       </c>
       <c r="K74" t="n">
         <v>1.833</v>
@@ -13507,10 +13507,10 @@
         <v>8.4</v>
       </c>
       <c r="J77" t="n">
-        <v>1.917</v>
+        <v>1.952</v>
       </c>
       <c r="K77" t="n">
-        <v>1.82</v>
+        <v>1.8</v>
       </c>
       <c r="L77" s="2" t="inlineStr">
         <is>
@@ -13699,10 +13699,10 @@
         <v>2.4</v>
       </c>
       <c r="J81" t="n">
-        <v>1.877</v>
+        <v>2.8</v>
       </c>
       <c r="K81" t="n">
-        <v>1.893</v>
+        <v>1.408</v>
       </c>
       <c r="L81" s="2" t="inlineStr">
         <is>
@@ -14179,10 +14179,10 @@
         <v>8</v>
       </c>
       <c r="J91" t="n">
-        <v>1.787</v>
+        <v>3.1</v>
       </c>
       <c r="K91" t="n">
-        <v>1.98</v>
+        <v>1.345</v>
       </c>
       <c r="L91" s="2" t="inlineStr">
         <is>
@@ -14227,10 +14227,10 @@
         <v>1.8</v>
       </c>
       <c r="J92" t="n">
-        <v>2.06</v>
+        <v>2.03</v>
       </c>
       <c r="K92" t="n">
-        <v>1.73</v>
+        <v>1.752</v>
       </c>
       <c r="L92" s="2" t="inlineStr">
         <is>
@@ -14275,10 +14275,10 @@
         <v>3.2</v>
       </c>
       <c r="J93" t="n">
-        <v>1.877</v>
+        <v>3.05</v>
       </c>
       <c r="K93" t="n">
-        <v>1.877</v>
+        <v>1.357</v>
       </c>
       <c r="L93" s="2" t="inlineStr">
         <is>
@@ -14323,10 +14323,10 @@
         <v>5</v>
       </c>
       <c r="J94" t="n">
-        <v>1.917</v>
+        <v>2.9</v>
       </c>
       <c r="K94" t="n">
-        <v>1.84</v>
+        <v>1.385</v>
       </c>
       <c r="L94" s="2" t="inlineStr">
         <is>
@@ -14371,10 +14371,10 @@
         <v>0.9</v>
       </c>
       <c r="J95" t="n">
-        <v>2.04</v>
+        <v>2.06</v>
       </c>
       <c r="K95" t="n">
-        <v>1.741</v>
+        <v>1.73</v>
       </c>
       <c r="L95" s="2" t="inlineStr">
         <is>
@@ -14419,10 +14419,10 @@
         <v>4.1</v>
       </c>
       <c r="J96" t="n">
-        <v>1.84</v>
+        <v>2.8</v>
       </c>
       <c r="K96" t="n">
-        <v>1.917</v>
+        <v>1.408</v>
       </c>
       <c r="L96" s="2" t="inlineStr">
         <is>
@@ -14467,10 +14467,10 @@
         <v>2.9</v>
       </c>
       <c r="J97" t="n">
-        <v>1.901</v>
+        <v>1.917</v>
       </c>
       <c r="K97" t="n">
-        <v>1.862</v>
+        <v>1.84</v>
       </c>
       <c r="L97" s="2" t="inlineStr">
         <is>
@@ -14515,10 +14515,10 @@
         <v>2.5</v>
       </c>
       <c r="J98" t="n">
-        <v>1.952</v>
+        <v>2.8</v>
       </c>
       <c r="K98" t="n">
-        <v>1.813</v>
+        <v>1.408</v>
       </c>
       <c r="L98" s="2" t="inlineStr">
         <is>
@@ -14563,10 +14563,10 @@
         <v>9.5</v>
       </c>
       <c r="J99" t="n">
-        <v>1.901</v>
+        <v>3</v>
       </c>
       <c r="K99" t="n">
-        <v>1.862</v>
+        <v>1.364</v>
       </c>
       <c r="L99" s="2" t="inlineStr">
         <is>
@@ -14611,10 +14611,10 @@
         <v>1.1</v>
       </c>
       <c r="J100" t="n">
-        <v>1.833</v>
+        <v>1.8</v>
       </c>
       <c r="K100" t="n">
-        <v>1.909</v>
+        <v>1.952</v>
       </c>
       <c r="L100" s="2" t="inlineStr">
         <is>
@@ -14659,10 +14659,10 @@
         <v>1.2</v>
       </c>
       <c r="J101" t="n">
-        <v>1.877</v>
+        <v>3.05</v>
       </c>
       <c r="K101" t="n">
-        <v>1.877</v>
+        <v>1.357</v>
       </c>
       <c r="L101" s="2" t="inlineStr">
         <is>
@@ -14707,10 +14707,10 @@
         <v>6.6</v>
       </c>
       <c r="J102" t="n">
-        <v>1.787</v>
+        <v>1.813</v>
       </c>
       <c r="K102" t="n">
-        <v>1.98</v>
+        <v>1.962</v>
       </c>
       <c r="L102" s="2" t="inlineStr">
         <is>
@@ -14755,10 +14755,10 @@
         <v>1</v>
       </c>
       <c r="J103" t="n">
-        <v>1.98</v>
+        <v>2.85</v>
       </c>
       <c r="K103" t="n">
-        <v>1.8</v>
+        <v>1.4</v>
       </c>
       <c r="L103" s="2" t="inlineStr">
         <is>
@@ -14803,10 +14803,10 @@
         <v>5.2</v>
       </c>
       <c r="J104" t="n">
-        <v>1.87</v>
+        <v>3.05</v>
       </c>
       <c r="K104" t="n">
-        <v>1.901</v>
+        <v>1.357</v>
       </c>
       <c r="L104" s="2" t="inlineStr">
         <is>
@@ -14899,10 +14899,10 @@
         <v>0</v>
       </c>
       <c r="J106" t="n">
-        <v>1.99</v>
+        <v>3.05</v>
       </c>
       <c r="K106" t="n">
-        <v>1.794</v>
+        <v>1.357</v>
       </c>
       <c r="L106" s="2" t="inlineStr">
         <is>
@@ -14947,10 +14947,10 @@
         <v>3.8</v>
       </c>
       <c r="J107" t="n">
-        <v>1.926</v>
+        <v>2.75</v>
       </c>
       <c r="K107" t="n">
-        <v>1.847</v>
+        <v>1.417</v>
       </c>
       <c r="L107" s="2" t="inlineStr">
         <is>
@@ -14995,10 +14995,10 @@
         <v>1.3</v>
       </c>
       <c r="J108" t="n">
-        <v>1.82</v>
+        <v>2.9</v>
       </c>
       <c r="K108" t="n">
-        <v>1.952</v>
+        <v>1.385</v>
       </c>
       <c r="L108" s="2" t="inlineStr">
         <is>
@@ -15043,10 +15043,10 @@
         <v>4.8</v>
       </c>
       <c r="J109" t="n">
-        <v>1.847</v>
+        <v>3.05</v>
       </c>
       <c r="K109" t="n">
-        <v>1.926</v>
+        <v>1.357</v>
       </c>
       <c r="L109" s="2" t="inlineStr">
         <is>
@@ -15091,10 +15091,10 @@
         <v>2.8</v>
       </c>
       <c r="J110" t="n">
-        <v>1.901</v>
+        <v>2.9</v>
       </c>
       <c r="K110" t="n">
-        <v>1.87</v>
+        <v>1.385</v>
       </c>
       <c r="L110" s="2" t="inlineStr">
         <is>
@@ -15187,10 +15187,10 @@
         <v>3.6</v>
       </c>
       <c r="J112" t="n">
-        <v>1.926</v>
+        <v>2.65</v>
       </c>
       <c r="K112" t="n">
-        <v>1.847</v>
+        <v>1.455</v>
       </c>
       <c r="L112" s="2" t="inlineStr">
         <is>
@@ -15235,10 +15235,10 @@
         <v>0.3</v>
       </c>
       <c r="J113" t="n">
-        <v>1.862</v>
+        <v>2.6</v>
       </c>
       <c r="K113" t="n">
-        <v>1.909</v>
+        <v>1.465</v>
       </c>
       <c r="L113" s="2" t="inlineStr">
         <is>
@@ -15283,10 +15283,10 @@
         <v>0.7</v>
       </c>
       <c r="J114" t="n">
-        <v>1.962</v>
+        <v>3</v>
       </c>
       <c r="K114" t="n">
-        <v>1.813</v>
+        <v>1.364</v>
       </c>
       <c r="L114" s="2" t="inlineStr">
         <is>
@@ -15331,10 +15331,10 @@
         <v>0.7</v>
       </c>
       <c r="J115" t="n">
-        <v>1.917</v>
+        <v>2.65</v>
       </c>
       <c r="K115" t="n">
-        <v>1.855</v>
+        <v>1.455</v>
       </c>
       <c r="L115" s="2" t="inlineStr">
         <is>

</xml_diff>